<commit_message>
feat: Add RCM and Scientific Inventory modules, optimize RBD functionality
- Add RCM key component configuration and calculation features
- Add Scientific Inventory management module
- Optimize RBD module failure rate units and calculation panel
- Update related API interfaces and route configurations
</commit_message>
<xml_diff>
--- a/apps/web-antd/public/产品零部件与备品对应关系配置.xlsx
+++ b/apps/web-antd/public/产品零部件与备品对应关系配置.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27948" windowHeight="12300"/>
+    <workbookView windowWidth="27948" windowHeight="12300" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="配置表" sheetId="1" r:id="rId1"/>
@@ -36,10 +36,10 @@
     <t>派生码</t>
   </si>
   <si>
-    <t>零部件名称（实际）</t>
+    <t>零部件名称（原装）</t>
   </si>
   <si>
-    <t>零部件物料编码（实际）</t>
+    <t>零部件物料编码（原装）</t>
   </si>
   <si>
     <t>零部件名称（备品）</t>
@@ -1339,7 +1339,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" s="1" customFormat="1" ht="86.4" spans="1:8">
+    <row r="2" s="1" customFormat="1" ht="43.2" spans="1:8">
       <c r="A2" s="5"/>
       <c r="B2" s="5"/>
       <c r="C2" s="5" t="s">
@@ -1359,7 +1359,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" ht="86.4" spans="3:8">
+    <row r="3" ht="43.2" spans="3:8">
       <c r="C3" s="1" t="s">
         <v>8</v>
       </c>

</xml_diff>